<commit_message>
Add batch 2 migration: 5 pages with images and updated infrastructure
- Migrated pages: family-and-visitor-resources, about-texas, medical-center,
  energy, entrepreneurship
- Added 49 local images across 5 page directories
- Updated content files with proper block structure and local image paths
- Added migration rules to Instructions.md
- Updated DEVELOPER-GUIDE.pdf with Adobe branding
- Removed obsolete markdown guides (replaced by PDF)
- Added import URL lists for batch 2

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-interior.report.xlsx
+++ b/tools/importer/reports/import-interior.report.xlsx
@@ -52,7 +52,7 @@
     <t>interior</t>
   </si>
   <si>
-    <t>2026-04-22T12:31:05.620Z</t>
+    <t>2026-05-06T12:32:50.043Z</t>
   </si>
   <si>
     <t>About | University of Texas at Austin</t>
@@ -157,7 +157,7 @@
     <t>energy</t>
   </si>
   <si>
-    <t>2026-04-22T12:31:09.685Z</t>
+    <t>2026-05-06T12:32:44.836Z</t>
   </si>
   <si>
     <t>Texas Energy | University of Texas at Austin</t>
@@ -172,7 +172,7 @@
     <t>entrepreneurship</t>
   </si>
   <si>
-    <t>2026-04-22T15:03:19.313Z</t>
+    <t>2026-05-06T12:32:54.596Z</t>
   </si>
   <si>
     <t>Texas Entrepreneurship | University of Texas at Austin</t>
@@ -205,7 +205,7 @@
     <t>family-and-visitor-resources</t>
   </si>
   <si>
-    <t>2026-04-22T10:58:44.407Z</t>
+    <t>2026-05-06T12:32:26.215Z</t>
   </si>
   <si>
     <t>Family and Visitor Resources | University of Texas at Austin</t>
@@ -253,7 +253,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-video","hero-video","cards-article","columns-promo","columns-impact","columns-impact","columns-impact","columns-outro"]</t>
+    <t>["hero-video","cards-article","columns-promo","columns-impact","columns-impact","columns-impact","columns-outro"]</t>
   </si>
   <si>
     <t>index</t>
@@ -262,7 +262,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-22T10:22:24.590Z</t>
+    <t>2026-04-26T11:24:55.843Z</t>
   </si>
   <si>
     <t>The University of Texas at Austin</t>
@@ -292,7 +292,7 @@
     <t>medical-center</t>
   </si>
   <si>
-    <t>2026-04-22T15:03:25.915Z</t>
+    <t>2026-05-06T12:32:39.072Z</t>
   </si>
   <si>
     <t>TEXAS Medical Center | University of Texas at Austin</t>

</xml_diff>